<commit_message>
Clarify Fleet Detailer as internal 2nd shift with 20-25 hrs
</commit_message>
<xml_diff>
--- a/Work_and_Travel_Master_Job_Database_2027.xlsx
+++ b/Work_and_Travel_Master_Job_Database_2027.xlsx
@@ -472,10 +472,10 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="114" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="132" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ทิป (Tips / Bonus)</t>
+          <t>ทิป ($/สัปดาห์)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -548,12 +548,12 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .00</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>ทิปหัวเตียง ~ -  / สัปดาห์</t>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>$15 - $30</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -563,12 +563,12 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR ตักไม่อั้น 7 วัน, รถรับส่งพนักงาน, ส่วนลดทัวร์/รถไฟ 50%</t>
+          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR ตักไม่อั้น 7 วัน, ทิปหัวเตียง, รถรับส่งพนักงาน, ส่วนลดทัวร์/รถไฟ 50%</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .00</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>ไม่มี ()</t>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -642,12 +642,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .00</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>ไม่มี (ได้กินอาหารในครัวฟรี)</t>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .50 / OT .25</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>💵 ทิปสดจากทัวร์ ~ -  / สัปดาห์</t>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>$40 - $70</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -704,12 +704,12 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, ได้ทิปเงินสดจากกรุ๊ปทัวร์ผู้สูงอายุ</t>
+          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, ทิปเงินสดจากกรุ๊ปทัวร์ผู้สูงอายุ</t>
         </is>
       </c>
     </row>
@@ -736,12 +736,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .50</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>🎁 โบนัส +.00/ชม. ท้ายทริป (ครบสัญญา)</t>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -751,12 +751,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$140</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>รถชัตเติลบัสขึ้น-ลงเขา Sugarloaf, ส่วนลดอาหารร้าน The Perk, วิวหุบเขาสวย</t>
+          <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป (ครบสัญญา), รถชัตเติลบัสขึ้น-ลงเขา Sugarloaf, ส่วนลดอาหารร้าน The Perk</t>
         </is>
       </c>
     </row>
@@ -783,12 +783,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .50 / OT .25</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>🎁 โบนัส +.00/ชม. ท้ายทริป (ครบสัญญา)</t>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -798,12 +798,12 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$140</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>โรงแรมหรู 4 ดาวบนยอดเขา, รถชัตเติลบัสรับส่ง, ส่วนลดอาหารห้องอาหาร Alpenglow</t>
+          <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป (ครบสัญญา), โรงแรมหรู 4 ดาว, รถชัตเติลบัส, ส่วนลดอาหารห้องอาหาร Alpenglow</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .00</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>💵 Tip Out สด ~ -  / คืน</t>
+          <t>ฐาน $14.00 / OT $21.00</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>$200 - $350</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -845,12 +845,12 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$140</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>โบนัส +.00/ชม. ท้ายทริป, ได้ทิปเงินสดจากแขกไฮเอนด์ร้านอาหารวิวพาโนรามา</t>
+          <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป, ทิปเงินสดจากแขกไฮเอนด์ร้านอาหารวิวพาโนรามา ($40-$70/คืน)</t>
         </is>
       </c>
     </row>
@@ -877,12 +877,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .00</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>ทิปหัวเตียง ~ -  / สัปดาห์</t>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>$10 - $20</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -892,12 +892,12 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, ชมวิวยอดเขาเดนาลี บรรยากาศสงบ ไม่กดดัน</t>
+          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, รถรับส่งพนักงาน, ชมวิวยอดเขาเดนาลี บรรยากาศสงบ</t>
         </is>
       </c>
     </row>
@@ -924,12 +924,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .50 / OT .25</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>ทิปเฉพาะ F&amp;B ~ -  / สัปดาห์</t>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>$20 - $40</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .75 / OT .62</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>ไม่มี (เน้นค่าแรงฐานสูงสุด)</t>
+          <t>ฐาน $17.75 / OT $26.62</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -986,12 +986,12 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> (หอพักฟรี!) + ค่าอาหาร EDR /wk</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>หอพักฟรี 100%, อาหารบุฟเฟต์ 3 มื้อ EDR, ส่วนลดซื้อของ 40%, เข้าอุทยาน Grand Teton &amp; Yellowstone ฟรี</t>
+          <t>หอพักฟรี 100%! + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), ส่วนลดซื้อของ 40%, เข้าอุทยาน Grand Teton &amp; Yellowstone ฟรี</t>
         </is>
       </c>
     </row>
@@ -1018,12 +1018,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .75 / OT .62</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>ไม่มี (กินฟรีในครัว)</t>
+          <t>ฐาน $17.75 / OT $26.62</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1033,12 +1033,12 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> (หอพักฟรี!) + ค่าอาหาร EDR /wk</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>หอพักฟรี 100%, อาหาร 3 มื้อ EDR + กินฟรีในครัว, สิทธิประโยชน์เครือ Vail Resorts</t>
+          <t>หอพักฟรี 100%! + อาหาร 3 มื้อ EDR + กินฟรีในครัว, สิทธิประโยชน์เครือ Vail Resorts</t>
         </is>
       </c>
     </row>
@@ -1065,12 +1065,12 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .70 / OT .55</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>ไม่มี ()</t>
+          <t>ฐาน $15.70 / OT $23.55</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1080,12 +1080,12 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์ (รวมหอพัก+อาหาร 3 มื้อ)</t>
+          <t>$120</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>หอพักใหม่ Arnica Development + บุฟเฟต์ 3 มื้อ EDR, เที่ยวบ่อน้ำพุร้อนและไกเซอร์ฟรี</t>
+          <t>รวมหอพัก + อาหารบุฟเฟต์ 3 มื้อ EDR, หอพักใหม่ Arnica, เที่ยวบ่อน้ำพุร้อนและไกเซอร์ Yellowstone ฟรี</t>
         </is>
       </c>
     </row>
@@ -1112,12 +1112,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .50 / OT .75</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>💵 ทิปสด ~ -  / สัปดาห์</t>
+          <t>ฐาน $16.50 / OT $24.75</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>$50 - $100</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$100</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>แคมป์กระโจมซาฟารีหรู, อาหารพนักงาน, แขกไฮเอนด์ ทิปเงินสดดี บรรยากาศเป็นกันเอง</t>
+          <t>แคมป์กระโจมซาฟารีหรู, อาหารพนักงาน, ทิปเงินสดจากแขกไฮเอนด์ บรรยากาศเป็นกันเอง</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1159,12 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .50</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>ไม่มี ()</t>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .00 – .00</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>💵 ทิปสด  -  / คืน</t>
+          <t>ฐาน $12.00 – $14.00</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>$250 - $500</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1221,12 +1221,12 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>ทำควบกับงานหลัก</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>รับทิปเงินสดทุกคืน ยัดกระเป๋ากลับห้องทันที, อาหารพนักงานในกะ</t>
+          <t>รับทิปเงินสดทุกคืน ยัดกระเป๋ากลับห้องทันที ($50-$100/คืน), อาหารพนักงานในกะ (ทำควบกับงานหลัก)</t>
         </is>
       </c>
     </row>
@@ -1253,12 +1253,12 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .50</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>ไม่มี (ปลอดภาษีรัฐ 0%)</t>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1268,12 +1268,12 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$110</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>นั่งรถราง Pigeon Forge Trolley -.50/วัน, บัตรเข้าสวนสนุก Dollywood &amp; Splash Country ฟรี</t>
+          <t>ปลอดภาษีเงินได้รัฐ 0%, นั่งรถราง Pigeon Forge Trolley $1-$2.50/วัน, บัตรเข้าสวนสนุก Dollywood &amp; Splash Country ฟรี</t>
         </is>
       </c>
     </row>
@@ -1300,12 +1300,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>ฐาน .00 / OT .00</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>ไม่มี (เน้นการันตี OT)</t>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1315,12 +1315,12 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$120</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>การันตีชั่วโมง OT สม่ำเสมอ ไม่ผันผวนตามนักท่องเที่ยว, อพาร์ตเมนต์แชร์กับเพื่อน</t>
+          <t>การันตีชั่วโมง OT สม่ำเสมอ 10-14 ชม./สัปดาห์ ไม่ผันผวนตามนักท่องเที่ยว, อพาร์ตเมนต์แชร์กับเพื่อน</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>ฐาน .50 / OT .75</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>ไม่มี ()</t>
+          <t>ฐาน $14.50 / OT $21.75</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> / สัปดาห์</t>
+          <t>$80</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>หอพักราคาถูกมาก (/wk), รถบัสรับส่งฟรี, บัตรเล่นเครื่องเล่นสวนสนุกระดับโลกฟรี</t>
+          <t>หอพักราคาถูกมาก ($80/wk), รถบัสรับส่งฟรี, บัตรเล่นเครื่องเล่นสวนสนุกระดับโลกฟรี</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Work Shifts schedule (Normal vs Peak) column
</commit_message>
<xml_diff>
--- a/Work_and_Travel_Master_Job_Database_2027.xlsx
+++ b/Work_and_Travel_Master_Job_Database_2027.xlsx
@@ -82,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -93,11 +93,17 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -464,18 +470,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="47" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="132" customWidth="1" min="9" max="9"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="132" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,25 +508,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>เวลาทำงานจริง (ช่วงปกติ / ช่วงพีค)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>ค่าแรงฐาน / OT ($/ชม.)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ทิป ($/สัปดาห์)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ชั่วโมงทำงานจริง (คิดเผื่อหัว-ท้ายซีซัน)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ค่าที่พัก ($/สัปดาห์)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>สวัสดิการ (อาหาร ฟรี หรือ อื่นๆ)</t>
         </is>
@@ -546,76 +558,88 @@
           <t>Housekeeping / Room Attendant</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:30 – 15:30 น. (8 ชม.)
+พีค: 07:00 – 17:30 น. (10 ชม. ควงกะ)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>$15 - $30</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>50 – 54 ชม./สัปดาห์ (พีค 58-62 ชม. / หัวท้าย 35-42 ชม.)</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR ตักไม่อั้น 7 วัน, ทิปหัวเตียง, รถรับส่งพนักงาน, ส่วนลดทัวร์/รถไฟ 50%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Denali Princess Wilderness Lodge</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Alaska (AK)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Acadex, OEG, IEE, Higher</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Motor Coach / Fleet Detailer (ล้างรถทัวร์กะดึก)</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Kitchen Stewarding / Dishwasher (ล้างจาน)</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 16:00 – 00:00 น. (8 ชม.)
+พีค: 15:00 – 01:30 น. (10.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>52 – 56 ชม./สัปดาห์ (กะดึก 21:00-02:00 OT ดกมาก)</t>
-        </is>
-      </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
+          <t>50 – 55 ชม./สัปดาห์ (ควงกะค่ำได้ง่าย)</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, กลางวันว่างนอนพักผ่อนหรือเดินป่าได้ทั้งวัน</t>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>อาหารบุฟเฟต์ 3 มื้อใน EDR + เชฟทำสเต๊ก/เบอร์เกอร์เลี้ยงในครัวฟรีทุกกะ</t>
         </is>
       </c>
     </row>
@@ -637,79 +661,91 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Kitchen Stewarding / Dishwasher (ล้างจาน)</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>ฐาน $16.00 / OT $24.00</t>
+          <t>Luggage Handler (พนักงานยกกระเป๋าทัวร์)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 น. หรือ 12:00 – 20:30 น.
+พีค: 07:00 – 18:30 น. (ตามรอบรถไฟ)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>$40 - $70</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>46 – 52 ชม./สัปดาห์</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, ทิปเงินสดจากกรุ๊ปทัวร์ผู้สูงอายุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Denali Princess Wilderness Lodge</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Alaska (AK)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>ขอทำเพิ่มหน้างาน (Internal 2nd Job)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Fleet Detailer (งานเสริมล้างรถทัวร์กะดึก)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 21:00 – 01:30 น. (4.5 ชม.)
+พีค: 21:00 – 02:30 น. (5.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>คิดเรต OT $24.00/ชม. ทันที</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>50 – 55 ชม./สัปดาห์ (ควงกะค่ำได้ง่าย)</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>$105</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>อาหารบุฟเฟต์ 3 มื้อใน EDR + เชฟทำสเต๊ก/เบอร์เกอร์เลี้ยงในครัวฟรีทุกกะ</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Denali Princess Wilderness Lodge</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Alaska (AK)</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Acadex, OEG, IEE, Higher</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Luggage Handler (พนักงานยกกระเป๋าทัวร์)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>ฐาน $15.50 / OT $23.25</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>$40 - $70</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>46 – 52 ชม./สัปดาห์</t>
-        </is>
-      </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>$105</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, ทิปเงินสดจากกรุ๊ปทัวร์ผู้สูงอายุ</t>
+          <t>20 – 25 ชม./สัปดาห์ (ทำควบหลังงานหลักแม่บ้าน)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>นับเป็นชั่วโมง OT $24.00 ทั้งหมด, ทำงานในอู่รถบัส Princess, อาหาร EDR 3 มื้อ</t>
         </is>
       </c>
     </row>
@@ -734,74 +770,86 @@
           <t>Housekeeping / Laundry</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 น. (8 ชม.)
+พีค: 08:00 – 17:00 น. (9 ชม.)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>40 – 45 ชม./สัปดาห์ (หัวท้าย 32-38 ชม.)</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>$140</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป (ครบสัญญา), รถชัตเติลบัสขึ้น-ลงเขา Sugarloaf, ส่วนลดอาหารร้าน The Perk</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Grande Denali Lodge</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Alaska (AK)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Acadex Thailand</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Housekeeping / Public Area Cleaner</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 น. (8 ชม.)
+พีค: 07:30 – 17:00 น. (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>42 – 46 ชม./สัปดาห์ (หัวท้าย 35-40 ชม.)</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>$140</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป (ครบสัญญา), โรงแรมหรู 4 ดาว, รถชัตเติลบัส, ส่วนลดอาหารห้องอาหาร Alpenglow</t>
         </is>
@@ -828,74 +876,86 @@
           <t>Busser / Food Runner (Alpenglow Restaurant)</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 16:30 – 22:30 น. (6 ชม.)
+พีค: 16:00 – 23:30 น. (7.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>ฐาน $14.00 / OT $21.00</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>$200 - $350</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>40 – 45 ชม./สัปดาห์</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>$140</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป, ทิปเงินสดจากแขกไฮเอนด์ร้านอาหารวิวพาโนรามา ($40-$70/คืน)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Mt. McKinley Princess Lodge</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Alaska (AK)</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Higher, OEG, Acadex</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Housekeeping / Kitchen / Laundry</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 น. (8 ชม.)
+พีค: 07:30 – 17:00 น. (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>$10 - $20</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>44 – 48 ชม./สัปดาห์ (หัวท้าย 35-40 ชม.)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, รถรับส่งพนักงาน, ชมวิวยอดเขาเดนาลี บรรยากาศสงบ</t>
         </is>
@@ -922,74 +982,86 @@
           <t>Food Runner / Laundry / Steward</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 06:30 – 14:30 น. หรือ 15:00 – 23:00 น.
+พีค: กะสลับตามรอบรถไฟ/เครื่องบิน 8 ชม.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>$20 - $40</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>36 – 40 ชม./สัปดาห์ (ไม่ค่อยมี OT)</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>หอพักในเมืองแฟร์แบงก์ส + รถชัตเติลบัส, ใกล้ Walmart และร้านอาหารไทย หางาน 2 ง่าย</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Grand Teton Lodge Company (GTLC)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Wyoming (WY)</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Acadex, Higher, OEG, IEE</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Housekeeping / Crew Member</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 น. (8 ชม.)
+พีค: 07:00 – 17:30 น. (10 ชม. ควงกะ)</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>ฐาน $17.75 / OT $26.62</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>54 – 60 ชม./สัปดาห์ (พีค 60-64 ชม. / หัวท้าย 40 ชม.)</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>หอพักฟรี 100%! + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), ส่วนลดซื้อของ 40%, เข้าอุทยาน Grand Teton &amp; Yellowstone ฟรี</t>
         </is>
@@ -1016,74 +1088,86 @@
           <t>Kitchen Crew / Dishwasher / Food Prep</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 06:00 – 14:30 น. หรือ 15:00 – 23:00 น.
+พีค: 14:00 – 00:30 น. (ช่วยจัดเลี้ยง Banquet)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>ฐาน $17.75 / OT $26.62</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>52 – 58 ชม./สัปดาห์ (ควงกะ Banquet ได้)</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>หอพักฟรี 100%! + อาหาร 3 มื้อ EDR + กินฟรีในครัว, สิทธิประโยชน์เครือ Vail Resorts</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Xanterra Yellowstone Lodges</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Wyoming/MT</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>OEG, IEE Thailand</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Hospitality Crew / Kitchen / Steward</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:00 – 15:30 น. หรือ 15:00 – 23:30 น.
+พีค: 06:30 – 16:30 น. (10 ชม.)</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>ฐาน $15.70 / OT $23.55</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>46 – 52 ชม./สัปดาห์ (หัวท้าย 38-42 ชม.)</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>$120</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>รวมหอพัก + อาหารบุฟเฟต์ 3 มื้อ EDR, หอพักใหม่ Arnica, เที่ยวบ่อน้ำพุร้อนและไกเซอร์ Yellowstone ฟรี</t>
         </is>
@@ -1110,74 +1194,86 @@
           <t>Housekeeping / Guest Service</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:30 – 16:30 น. (8 ชม.)
+พีค: 08:00 – 17:30 น. (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>ฐาน $16.50 / OT $24.75</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>$50 - $100</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>42 – 46 ชม./สัปดาห์</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>$100</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>แคมป์กระโจมซาฟารีหรู, อาหารพนักงาน, ทิปเงินสดจากแขกไฮเอนด์ บรรยากาศเป็นกันเอง</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Kalahari Resorts &amp; Conventions</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Wisconsin (WI)</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>OEG, Acadex, Higher</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Lifeguard / Housekeeping (งานหลัก)</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 น. หรือ 12:00 – 20:30 น.
+พีค: 09:00 – 19:30 น. (10 ชม.)</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>38 – 44 ชม./สัปดาห์ (เกลี่ยกะ 40 ชม.)</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>หอพัก Kalahari Village, บัตรเล่นสวนน้ำฟรี, เมืองปั่นจักรยาน 100%, หางาน 2 ร้านอาหารง่าย</t>
         </is>
@@ -1204,74 +1300,86 @@
           <t>Barback / Busser / Runner (งานที่สอง)</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 17:30 – 22:30 น. (5 ชม.)
+พีค: 17:00 – 00:30 น. (7.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>ฐาน $12.00 – $14.00</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>$250 - $500</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>20 – 25 ชม./สัปดาห์ (กะค่ำ 17:30-23:00)</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>รับทิปเงินสดทุกคืน ยัดกระเป๋ากลับห้องทันที ($50-$100/คืน), อาหารพนักงานในกะ (ทำควบกับงานหลัก)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Dollywood Theme Park &amp; Resorts</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Tennessee (TN)</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>New Step, Acadex</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Ride Operator / Food Service / Retail</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 น. (8 ชม.)
+พีค: 09:00 – 21:30 น. (12 ชม. สวนสนุกเปิดดึก)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>44 – 50 ชม./สัปดาห์ (หัวท้าย 35-40 ชม.)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>$110</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>ปลอดภาษีเงินได้รัฐ 0%, นั่งรถราง Pigeon Forge Trolley $1-$2.50/วัน, บัตรเข้าสวนสนุก Dollywood &amp; Splash Country ฟรี</t>
         </is>
@@ -1298,74 +1406,86 @@
           <t>Pool Lifeguard</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 10:30 – 19:30 น. (9 ชม.)
+พีค: 10:00 – 20:30 น. (10.5 ชม. สระเปิดยาว)</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>50 – 54 ชม./สัปดาห์ (การันตี OT 10-14 ชม.)</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>$120</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>การันตีชั่วโมง OT สม่ำเสมอ 10-14 ชม./สัปดาห์ ไม่ผันผวนตามนักท่องเที่ยว, อพาร์ตเมนต์แชร์กับเพื่อน</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Cedar Point Amusement Park</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Ohio (OH)</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>OEG, IEE Thailand</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Ride Operator / Food Service</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 10:00 – 18:30 น. (8 ชม.)
+พีค: 09:30 – 22:30 น. (12 ชม. สวนสนุกปิดดึก)</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>ฐาน $14.50 / OT $21.75</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>46 – 52 ชม./สัปดาห์ (หัวท้าย 38-42 ชม.)</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>$80</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>หอพักราคาถูกมาก ($80/wk), รถบัสรับส่งฟรี, บัตรเล่นเครื่องเล่นสวนสนุกระดับโลกฟรี</t>
         </is>

</xml_diff>

<commit_message>
Verified and integrated all 6 major Thai agencies (OEG, Acadex, IEE, IEO, New Step, Higher) across 38 Tier S-A employers
</commit_message>
<xml_diff>
--- a/Work_and_Travel_Master_Job_Database_2027.xlsx
+++ b/Work_and_Travel_Master_Job_Database_2027.xlsx
@@ -499,13 +499,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
@@ -530,7 +530,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Agency ที่ถือสัญญา</t>
+          <t>Agency ที่ถือสัญญา (ครบ 6 แห่ง)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Acadex, OEG, IEE, Higher</t>
+          <t>Acadex, OEG, IEE, Higher, IEO</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Acadex, OEG, IEE, Higher</t>
+          <t>Acadex, OEG, IEE, Higher, IEO</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Acadex Thailand</t>
+          <t>Acadex Thailand, IEO</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Higher, OEG, Acadex</t>
+          <t>Higher, OEG, Acadex, IEO</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>IEE, Acadex, Higher</t>
+          <t>IEE, Acadex, Higher, IEO</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>OEG, Acadex, ALC</t>
+          <t>OEG, Acadex, ALC, IEO</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>OEG, Acadex, Higher</t>
+          <t>OEG, Acadex, Higher, IEO</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>OEG, Higher</t>
+          <t>OEG, Higher, Acadex</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Higher, IEE, Acadex</t>
+          <t>Higher, IEE, Acadex, IEO</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Acadex, Higher, OEG, IEE</t>
+          <t>Acadex, Higher, OEG, IEE, IEO</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Acadex, Higher, OEG, IEE</t>
+          <t>Acadex, Higher, OEG, IEE, IEO</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Higher, Acadex</t>
+          <t>Higher, Acadex, IEO</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>OEG, IEE Thailand</t>
+          <t>OEG, IEE Thailand, IEO</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>OEG, Acadex</t>
+          <t>OEG, Acadex, IEO</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Acadex, OEG</t>
+          <t>Acadex, OEG, IEO</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Higher Education</t>
+          <t>Higher Education, IEO</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>OEG, Acadex, Higher</t>
+          <t>OEG, Acadex, Higher, IEO, New Step</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>OEG, IEE, Acadex</t>
+          <t>OEG, IEE, Acadex, IEO</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>New Step, Acadex, Higher</t>
+          <t>New Step, Acadex, Higher, IEO</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>OEG, IEE, New Step</t>
+          <t>OEG, IEE, New Step, IEO</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Higher, Acadex, IEE</t>
+          <t>Higher, Acadex, IEE, IEO</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Acadex, OEG</t>
+          <t>Acadex, OEG, IEO</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>New Step, Acadex</t>
+          <t>New Step, Acadex, IEO</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>New Step, Acadex</t>
+          <t>New Step, Acadex, IEO</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>OEG, Acadex, Higher</t>
+          <t>OEG, Acadex, Higher, IEO</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Higher, IEE</t>
+          <t>Higher, IEE, IEO</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>IEE, New Step</t>
+          <t>IEE, New Step, IEO</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>OEG, Acadex, IEE</t>
+          <t>OEG, Acadex, IEE, IEO</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>OEG, Acadex</t>
+          <t>OEG, Acadex, IEO</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>New Step, Higher, IEE</t>
+          <t>New Step, Higher, IEE, IEO</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>OEG, New Step</t>
+          <t>OEG, New Step, IEO</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>OEG, Acadex, Higher</t>
+          <t>OEG, Acadex, Higher, IEO</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>OEG, Acadex</t>
+          <t>OEG, Acadex, IEO</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Acadex, Higher, IEE</t>
+          <t>Acadex, Higher, IEE, IEO</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2899,1222 +2899,1494 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
+          <t>Tier A - Florida (FL)</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Universal Orlando Resort &amp; Volcano Bay</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>OEG, IEE, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Attractions Attendant / Culinary / Lifeguard</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 (8 ชม.)
+พีค: 09:00 – 22:00 (12 ชม.)</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>42 – 48 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>$130</t>
+        </is>
+      </c>
+      <c r="J36" s="10" t="inlineStr">
+        <is>
+          <t>สวนสนุกระดับโลก ยูนิเวอร์แซล ออร์แลนโด, ปลอดภาษีเงินได้รัฐ 0%, บัตรเข้าสวนสนุกฟรี</t>
+        </is>
+      </c>
+      <c r="K36" s="10" t="inlineStr">
+        <is>
+          <t>🎸 Universal CityWalk Eateries: Food Runner/Busser บาร์ดึก 18:30-01:00 น. (ทิปสด $60-$100/คืน)</t>
+        </is>
+      </c>
+      <c r="L36" s="10" t="inlineStr">
+        <is>
+          <t>🍔 The Cowfish Sushi Burger Bar: ล้างจาน/ผู้ช่วยครัว 19:00-01:00 น. ($15/ชม. + ทิป)</t>
+        </is>
+      </c>
+      <c r="M36" s="10" t="inlineStr">
+        <is>
+          <t>🍕 Red Oven Pizza Bakery: ผู้ช่วยทำพิซซ่ากะดึก 18:30-00:30 น.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Tier A - Florida (FL)</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Busch Gardens Tampa Bay &amp; Adventure Island</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>New Step, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Ride Operator / Lifeguard / Food Service</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 (8 ชม.)
+พีค: 09:00 – 21:30 (11.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>42 – 48 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>$120</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>สวนสนุกโรลเลอร์โคสเตอร์อันดับ 1 ในแทมปาและสวนน้ำ, ปลอดภาษีรัฐ 0%</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>🍺 Ybor City Historic Bars (แทมปา): Barback ผับประวัติศาสตร์ 19:00-01:30 น. (ทิปสด $60-$110/คืน)</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
+          <t>🦀 Columbia Restaurant (ร้านสเปนชื่อดังที่สุด): Busser 18:30-23:30 น. (ทิปดี)</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>🍔 Portillo’s Hot Dogs Tampa: ครัว/แคชเชียร์รอบดึก 18:30-00:00 น. ($15/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Tier A - Florida (FL)</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Gaylord Palms Resort &amp; Convention Center (Kissimmee)</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>OEG, Acadex, Higher</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Housekeeping / Banquet Server / Steward</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 (8 ชม.)
+พีค: 07:30 – 17:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>$20 - $50</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>44 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>$125</t>
+        </is>
+      </c>
+      <c r="J38" s="10" t="inlineStr">
+        <is>
+          <t>รีสอร์ตศูนย์ประชุมโดมกระจกยักษ์ระดับ 4 ดาว Marriott, ปลอดภาษีรัฐ 0%</t>
+        </is>
+      </c>
+      <c r="K38" s="10" t="inlineStr">
+        <is>
+          <t>🥩 Old Hickory Steakhouse (ในรีสอร์ต): Busser ร้านสเต๊กหรู 17:30-23:00 น. (ทิปสด $70-$120)</t>
+        </is>
+      </c>
+      <c r="L38" s="10" t="inlineStr">
+        <is>
+          <t>🌴 Wreckers Sports Bar (ในรีสอร์ต): Barback ผับกีฬาจอ 2 ชั้น 18:30-00:30 น. (ขอ OT ในรีสอร์ต $24/ชม.)</t>
+        </is>
+      </c>
+      <c r="M38" s="10" t="inlineStr">
+        <is>
+          <t>🛍️ Disney Springs Eateries: Food Runner ร้านอาหารฝั่งดิสนีย์ 19:00-01:00 น.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
           <t>Tier A - Maryland (MD)</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Premier Aquatics / High Sierra Pools (Bethesda/Rockville)</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Acadex, New Step, ALC</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Acadex, New Step, ALC, IEO</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Pool Lifeguard</t>
         </is>
       </c>
-      <c r="E36" s="10" t="inlineStr">
+      <c r="E39" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 10:30 – 19:30 (9 ชม.)
 พีค: 10:00 – 20:30 (10.5 ชม. สระเปิดยาว)</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="G36" s="8" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H36" s="8" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>50 – 54 ชม./wk (การันตี OT)</t>
         </is>
       </c>
-      <c r="I36" s="8" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>$120</t>
         </is>
       </c>
-      <c r="J36" s="10" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
         <is>
           <t>การันตีชั่วโมง OT แน่นอนสัปดาห์ละ 10-14 ชม., อพาร์ตเมนต์แชร์กับเพื่อน, รถไฟใต้ดิน Metro เข้า DC</t>
         </is>
       </c>
-      <c r="K36" s="10" t="inlineStr">
+      <c r="K39" s="7" t="inlineStr">
         <is>
           <t>🛒 Giant Food / Safeway: พนักงานจัดสต็อกสินค้ากะดึก 20:30-01:00 น. ($16-$17.50/ชม. มีสาขาใกล้ที่พัก)</t>
         </is>
       </c>
-      <c r="L36" s="10" t="inlineStr">
+      <c r="L39" s="7" t="inlineStr">
         <is>
           <t>🍜 Thai Tanic / Ruan Thai: ผู้ช่วยครัว/แพ็กอาหาร 20:00-23:30 น. (มีอาหารไทยฟรี)</t>
         </is>
       </c>
-      <c r="M36" s="10" t="inlineStr">
+      <c r="M39" s="7" t="inlineStr">
         <is>
           <t>🎯 Target / CVS Pharmacy: แคชเชียร์/ปิดร้าน 20:00-23:30 น. ($16.00/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Tier A - Maryland (MD)</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>Ocean City Boardwalk Hotels &amp; Resorts</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>IEE, New Step, OEG</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>IEE, New Step, OEG, IEO</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>Housekeeping / Ride Operator</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E40" s="10" t="inlineStr">
         <is>
           <t>ปกติ: 08:30 – 16:30 (8 ชม.)
 พีค: 08:00 – 17:30 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F40" s="8" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G40" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="H40" s="8" t="inlineStr">
         <is>
           <t>44 – 50 ชม./wk</t>
         </is>
       </c>
-      <c r="I37" s="5" t="inlineStr">
+      <c r="I40" s="8" t="inlineStr">
         <is>
           <t>$125</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
+      <c r="J40" s="10" t="inlineStr">
         <is>
           <t>เมืองตากอากาศชายหาด Atlantic, รถบัส Coastal Highway วิ่ง 24 ชม., หางานสองง่ายมาก</t>
         </is>
       </c>
-      <c r="K37" s="7" t="inlineStr">
+      <c r="K40" s="10" t="inlineStr">
         <is>
           <t>🌴 Seacrets Jamaica USA (ผับริมหาดยักษ์ใหญ่): Barback/Busser 18:00-01:30 น. ($12/ชม. + ทิปสดมหาศาล $80-$150/คืน)</t>
         </is>
       </c>
-      <c r="L37" s="7" t="inlineStr">
+      <c r="L40" s="10" t="inlineStr">
         <is>
           <t>🍟 Thrasher’s French Fries (ริมหาด): แคชเชียร์/ทอดเฟรนช์ฟรายส์ 18:00-23:00 น. ($15/ชม.)</t>
         </is>
       </c>
-      <c r="M37" s="7" t="inlineStr">
+      <c r="M40" s="10" t="inlineStr">
         <is>
           <t>🍺 Shenanigans Irish Pub: ล้างจาน/ผู้ช่วยบาร์ 18:30-00:30 น. ($14/ชม. + ทิป)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>Tier A - Maryland (MD)</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>Jolly Roger Amusement Park &amp; Splash Mountain (Ocean City)</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>New Step, IEE</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>New Step, IEE, IEO</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Ride Operator / Lifeguard / Park Services</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 11:00 – 19:00 (8 ชม.)
 พีค: 10:00 – 23:00 (12 ชม.)</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="G38" s="8" t="inlineStr">
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H38" s="8" t="inlineStr">
+      <c r="H41" s="5" t="inlineStr">
         <is>
           <t>45 – 52 ชม./wk</t>
         </is>
       </c>
-      <c r="I38" s="8" t="inlineStr">
+      <c r="I41" s="5" t="inlineStr">
         <is>
           <t>$120</t>
         </is>
       </c>
-      <c r="J38" s="10" t="inlineStr">
+      <c r="J41" s="7" t="inlineStr">
         <is>
           <t>สวนสนุกและสวนน้ำที่ใหญ่ที่สุดใน Ocean City, เล่นสวนสนุกฟรี, มีรถเมล์ผ่านหน้าสวนสนุก</t>
         </is>
       </c>
-      <c r="K38" s="10" t="inlineStr">
+      <c r="K41" s="7" t="inlineStr">
         <is>
           <t>🦀 Higgins Crab House: Busser ร้านปูยักษ์ 19:30-00:30 น. ($13/ชม. + ทิปสด $60-$90/คืน)</t>
         </is>
       </c>
-      <c r="L38" s="10" t="inlineStr">
+      <c r="L41" s="7" t="inlineStr">
         <is>
           <t>🍕 Dough Roller Pizza (Boardwalk): ล้างจาน/ทำพิซซ่ากะดึก 19:30-01:00 น. ($15/ชม.)</t>
         </is>
       </c>
-      <c r="M38" s="10" t="inlineStr">
+      <c r="M41" s="7" t="inlineStr">
         <is>
           <t>🍦 Dumser’s Dairyland: ตักไอศกรีม/แคชเชียร์ 19:00-23:30 น. ($15/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Tier A - Virginia (VA)</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>Busch Gardens Williamsburg &amp; Water Country USA</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>New Step, Acadex</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>New Step, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
         <is>
           <t>Ride Operator / Culinary Operations</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>ปกติ: 09:30 – 18:00 (8 ชม.)
 พีค: 09:00 – 21:30 (12 ชม. สวนสนุกเปิดดึก)</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t>ฐาน $14.50 / OT $21.75</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G42" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="H42" s="8" t="inlineStr">
         <is>
           <t>44 – 50 ชม./wk</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="I42" s="8" t="inlineStr">
         <is>
           <t>$115</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr">
+      <c r="J42" s="10" t="inlineStr">
         <is>
           <t>สวนสนุกธีมยุโรปชื่อดัง, บัตรเข้าสวนสนุกและสวนน้ำฟรี, หอพักพนักงาน Williamsburg</t>
         </is>
       </c>
-      <c r="K39" s="7" t="inlineStr">
+      <c r="K42" s="10" t="inlineStr">
         <is>
           <t>🏰 Kingsmill Resort (ริมแม่น้ำ James River): Banquet Server/Busser งานจัดเลี้ยง 18:30-23:00 น. (ทิปสด $50-$90/คืน)</t>
         </is>
       </c>
-      <c r="L39" s="7" t="inlineStr">
+      <c r="L42" s="10" t="inlineStr">
         <is>
           <t>🦀 Captain George’s Seafood Buffet: Busser/Dishwasher บุฟเฟต์ซีฟู้ดยักษ์ใหญ่ 18:30-23:30 น. (คนแน่นมาก ทิปดี)</t>
         </is>
       </c>
-      <c r="M39" s="7" t="inlineStr">
+      <c r="M42" s="10" t="inlineStr">
         <is>
           <t>🥞 Cracker Barrel / Pancake House: ผู้ช่วยครัว/ล้างจานรอบค่ำ 18:00-22:00 น. ($14.50/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>Tier A - Virginia (VA)</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Virginia Beach Oceanfront Resorts &amp; Boardwalk</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>IEE, New Step, Acadex</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>IEE, New Step, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Housekeeping / Beach Attendant</t>
         </is>
       </c>
-      <c r="E40" s="10" t="inlineStr">
+      <c r="E43" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 08:30 – 16:30 (8 ชม.)
 พีค: 08:00 – 17:30 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
+      <c r="F43" s="5" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="G40" s="8" t="inlineStr">
+      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>$15 - $30</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr">
+      <c r="H43" s="5" t="inlineStr">
         <is>
           <t>42 – 48 ชม./wk</t>
         </is>
       </c>
-      <c r="I40" s="8" t="inlineStr">
+      <c r="I43" s="5" t="inlineStr">
         <is>
           <t>$130</t>
         </is>
       </c>
-      <c r="J40" s="10" t="inlineStr">
+      <c r="J43" s="7" t="inlineStr">
         <is>
           <t>เมืองตากอากาศชายทะเลเวอร์จิเนีย มีทางเดินเลียบหาดยาว 3 ไมล์, รถราง Wave Trolley สะดวก</t>
         </is>
       </c>
-      <c r="K40" s="10" t="inlineStr">
+      <c r="K43" s="7" t="inlineStr">
         <is>
           <t>🍺 Waterman’s Surfside Grille: Barback/Busser ร้านริมหาดคนแน่น 18:00-00:30 น. (ทิปสด $70-$120/คืน)</t>
         </is>
       </c>
-      <c r="L40" s="10" t="inlineStr">
+      <c r="L43" s="7" t="inlineStr">
         <is>
           <t>🦀 Catch 31 Fish Bar: Food Runner/Busser 18:00-23:30 น. (ทิปดี)</t>
         </is>
       </c>
-      <c r="M40" s="10" t="inlineStr">
+      <c r="M43" s="7" t="inlineStr">
         <is>
           <t>🍕 Dough Boy’s California Pizza: ผู้ช่วยครัว/ล้างจาน 18:30-00:00 น. ($14.50/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Tier A - New Jersey (NJ)</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Morey’s Piers &amp; Beachfront Waterparks (Wildwood, NJ)</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>OEG, IEE, New Step, IEO</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Ride Operator / Lifeguard / Pier Services</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 11:00 – 19:00 (8 ชม.)
+พีค: 10:30 – 23:30 (12 ชม.)</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>45 – 52 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>$120</t>
+        </is>
+      </c>
+      <c r="J44" s="10" t="inlineStr">
+        <is>
+          <t>สวนสนุกริมสะพานปลาชานหาดที่ใหญ่ที่สุดในฝั่ง East Coast, เล่นเครื่องเล่นฟรี, เมืองจักรยาน</t>
+        </is>
+      </c>
+      <c r="K44" s="10" t="inlineStr">
+        <is>
+          <t>🍕 Mack’s Pizza / Sam’s Pizza (Boardwalk): ล้างจาน/ทำพิซซ่ากะดึก 19:30-01:30 น. ($15/ชม.)</t>
+        </is>
+      </c>
+      <c r="L44" s="10" t="inlineStr">
+        <is>
+          <t>🍺 The Wharf Restaurant &amp; Bar: Barback/Busser ร้านอาหารริมน้ำ 19:00-01:00 น. (ทิปสด $70-$120/คืน)</t>
+        </is>
+      </c>
+      <c r="M44" s="10" t="inlineStr">
+        <is>
+          <t>🍦 Curley’s Fries / Kohr Brothers: แคชเชียร์/ตักไอศกรีม 19:00-23:30 น. ($15.50/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>Tier A - South Dakota (SD)</t>
         </is>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Xanterra Mount Rushmore / Keystone Lodges</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>OEG, IEE, Higher</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>OEG, IEE, Higher, IEO</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Retail / Food Service / Housekeeping</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="E45" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 08:30 – 16:30 (8 ชม.)
 พีค: 08:00 – 17:30 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>44 – 50 ชม./wk</t>
         </is>
       </c>
-      <c r="I41" s="5" t="inlineStr">
+      <c r="I45" s="5" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="J41" s="7" t="inlineStr">
+      <c r="J45" s="7" t="inlineStr">
         <is>
           <t>ทำงานหน้าอนุสรณ์สถานแห่งชาติ Mount Rushmore, ปลอดภาษีรัฐ 0%, หอพัก+อาหาร EDR</t>
         </is>
       </c>
-      <c r="K41" s="7" t="inlineStr">
+      <c r="K45" s="7" t="inlineStr">
         <is>
           <t>🍔 Carver’s Cafe at Mt Rushmore: ล้างจาน/ปิดครัว 17:00-21:30 น. (ขอ OT ในอุทยาน $23.25/ชม.)</t>
         </is>
       </c>
-      <c r="L41" s="7" t="inlineStr">
+      <c r="L45" s="7" t="inlineStr">
         <is>
           <t>🥩 Ruby House Restaurant (Keystone): Busser ร้านอาหารธีมคาวบอยย้อนยุค 17:30-22:30 น. ($13/ชม. + ทิป)</t>
         </is>
       </c>
-      <c r="M41" s="7" t="inlineStr">
+      <c r="M45" s="7" t="inlineStr">
         <is>
           <t>🚂 1880 Train / Keystone Gift Shops: พนักงานร้านของฝาก/สถานีรถไฟโบราณ 17:00-21:30 น. ($15/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>Tier A - South Dakota (SD)</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B46" s="9" t="inlineStr">
         <is>
           <t>Custer State Park Resorts (State Game Lodge / Sylvan)</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>Higher, Acadex</t>
-        </is>
-      </c>
-      <c r="D42" s="9" t="inlineStr">
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Higher, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
         <is>
           <t>Guest Service / Housekeeping</t>
         </is>
       </c>
-      <c r="E42" s="10" t="inlineStr">
+      <c r="E46" s="10" t="inlineStr">
         <is>
           <t>ปกติ: 07:30 – 15:30 (8 ชม.)
 พีค: 07:00 – 16:30 (9 ชม.)</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
+      <c r="F46" s="8" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="G42" s="8" t="inlineStr">
+      <c r="G46" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H42" s="8" t="inlineStr">
+      <c r="H46" s="8" t="inlineStr">
         <is>
           <t>42 – 48 ชม./wk</t>
         </is>
       </c>
-      <c r="I42" s="8" t="inlineStr">
+      <c r="I46" s="8" t="inlineStr">
         <is>
           <t>$105 (รวมกิน)</t>
         </is>
       </c>
-      <c r="J42" s="10" t="inlineStr">
+      <c r="J46" s="10" t="inlineStr">
         <is>
           <t>อุทยานธรรมชาติฝูงควายไบซัน Custer SP, ปลอดภาษีรัฐ 0%, หอพัก+อาหาร EDR</t>
         </is>
       </c>
-      <c r="K42" s="10" t="inlineStr">
+      <c r="K46" s="10" t="inlineStr">
         <is>
           <t>🥩 State Game Lodge Dining Room: Busser ร้านสเต๊กควายไบซันหรู 17:00-22:00 น. ($13/ชม. + ทิปสด $50-$80)</t>
         </is>
       </c>
-      <c r="L42" s="10" t="inlineStr">
+      <c r="L46" s="10" t="inlineStr">
         <is>
           <t>🍔 Black Hills Burger &amp; Bun (เมือง Custer): ล้างจาน/ครัว 17:00-21:30 น. ($15/ชม. + กินฟรี)</t>
         </is>
       </c>
-      <c r="M42" s="10" t="inlineStr">
+      <c r="M46" s="10" t="inlineStr">
         <is>
           <t>🏕️ Sylvan Lake General Store: พนักงานมินิมาร์ท/เช่าเรือแคนู 16:30-21:00 น.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>Tier A - South Dakota (SD)</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>Wall Drug Store (Wall, SD)</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>IEE, Acadex</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>IEE, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Retail / Restaurant Staff / Fast Food</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 08:00 – 16:30 (8 ชม.)
 พีค: 07:30 – 17:30 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr">
+      <c r="H47" s="5" t="inlineStr">
         <is>
           <t>45 – 50 ชม./wk</t>
         </is>
       </c>
-      <c r="I43" s="5" t="inlineStr">
+      <c r="I47" s="5" t="inlineStr">
         <is>
           <t>$85 (ถูกมาก)</t>
         </is>
       </c>
-      <c r="J43" s="7" t="inlineStr">
+      <c r="J47" s="7" t="inlineStr">
         <is>
           <t>ห้างคาวบอยระดับตำนานของอเมริกา จุดแวะพักยอดฮิตก่อนเข้า Badlands NP, หอพักราคาถูก</t>
         </is>
       </c>
-      <c r="K43" s="7" t="inlineStr">
+      <c r="K47" s="7" t="inlineStr">
         <is>
           <t>☕ Wall Drug Western Art Dining Room: Busser/Steward 17:00-22:00 น. (ขอ OT ในตัว $23.25)</t>
         </is>
       </c>
-      <c r="L43" s="7" t="inlineStr">
+      <c r="L47" s="7" t="inlineStr">
         <is>
           <t>🍩 Wall Drug Famous Donut Kitchen: ช่วยทำโดนัท/เบเกอรี่รอบเย็น 16:30-21:00 น.</t>
         </is>
       </c>
-      <c r="M43" s="7" t="inlineStr">
+      <c r="M47" s="7" t="inlineStr">
         <is>
           <t>🌵 Badlands Saloon &amp; Grille: Barback/ล้างจาน 18:00-23:00 น. ($14.50/ชม. + ทิป)</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>Tier A - South Dakota (SD)</t>
         </is>
       </c>
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>Deadwood Historic Hotels &amp; Casinos (The Lodge at Deadwood)</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>Higher, New Step</t>
-        </is>
-      </c>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Higher, New Step, IEO</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
         <is>
           <t>Housekeeping / Food &amp; Beverage</t>
         </is>
       </c>
-      <c r="E44" s="10" t="inlineStr">
+      <c r="E48" s="10" t="inlineStr">
         <is>
           <t>ปกติ: 08:00 – 16:30 (8 ชม.)
 พีค: 07:30 – 17:00 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
+      <c r="F48" s="8" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="G44" s="8" t="inlineStr">
+      <c r="G48" s="8" t="inlineStr">
         <is>
           <t>$20 - $50</t>
         </is>
       </c>
-      <c r="H44" s="8" t="inlineStr">
+      <c r="H48" s="8" t="inlineStr">
         <is>
           <t>42 – 48 ชม./wk</t>
         </is>
       </c>
-      <c r="I44" s="8" t="inlineStr">
+      <c r="I48" s="8" t="inlineStr">
         <is>
           <t>$100</t>
         </is>
       </c>
-      <c r="J44" s="10" t="inlineStr">
+      <c r="J48" s="10" t="inlineStr">
         <is>
           <t>เมืองคาวบอยคาสิโนประวัติศาสตร์ ปลอดภาษีรัฐ 0%, มีรถราง Deadwood Trolley $1</t>
         </is>
       </c>
-      <c r="K44" s="10" t="inlineStr">
+      <c r="K48" s="10" t="inlineStr">
         <is>
           <t>🥩 Deadwood Grille / O’Shea’s: Busser/Runner 17:30-23:00 น. ($13/ชม. + ทิปสด $50-$90/คืน)</t>
         </is>
       </c>
-      <c r="L44" s="10" t="inlineStr">
+      <c r="L48" s="10" t="inlineStr">
         <is>
           <t>🎰 Mineral Palace / Silverado Casino: Barback บาร์ในคาสิโน 18:30-01:00 น. (ทิปดี)</t>
         </is>
       </c>
-      <c r="M44" s="10" t="inlineStr">
+      <c r="M48" s="10" t="inlineStr">
         <is>
           <t>🍕 Mustang Sally’s Sports Bar: ผู้ช่วยครัว/ล้างจาน 18:00-00:00 น. ($14.50/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Tier A - Utah (UT)</t>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>Zion National Park Lodge (Xanterra Springdale)</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>OEG, IEE, Acadex</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>OEG, IEE, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Hospitality Crew / Housekeeping</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 07:30 – 15:30 (8 ชม.)
 พีค: 07:00 – 16:30 (9 ชม.)</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F49" s="5" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H45" s="5" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>44 – 50 ชม./wk</t>
         </is>
       </c>
-      <c r="I45" s="5" t="inlineStr">
+      <c r="I49" s="5" t="inlineStr">
         <is>
           <t>$110</t>
         </is>
       </c>
-      <c r="J45" s="7" t="inlineStr">
+      <c r="J49" s="7" t="inlineStr">
         <is>
           <t>อุทยานแห่งชาติหุบเขาผาแดง Zion NP, มีรถชัตเติลบัสฟรีวิ่งตลอดถนน Springdale</t>
         </is>
       </c>
-      <c r="K45" s="7" t="inlineStr">
+      <c r="K49" s="7" t="inlineStr">
         <is>
           <t>🌮 Bit &amp; Spur Restaurant &amp; Saloon: Busser/Barback 17:30-23:00 น. ($13/ชม. + ทิปสดแขกต่างชาติ $50-$90/คืน)</t>
         </is>
       </c>
-      <c r="L45" s="7" t="inlineStr">
+      <c r="L49" s="7" t="inlineStr">
         <is>
           <t>🍔 Oscar’s Cafe (Springdale): Food Runner/Busser 17:00-22:00 น. ($13/ชม. + ทิป)</t>
         </is>
       </c>
-      <c r="M45" s="7" t="inlineStr">
+      <c r="M49" s="7" t="inlineStr">
         <is>
           <t>🍺 Zion Canyon Brew Pub: ล้างจาน/ผู้ช่วยครัวหน้าปากทางเข้าอุทยาน 18:00-23:30 น. ($15/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Tier A - Utah (UT)</t>
         </is>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>Ruby’s Inn / Bryce Canyon Grand Hotel</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>Higher, IEE, Acadex</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Higher, IEE, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
         <is>
           <t>Housekeeping / Fast Food / Retail</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
+      <c r="E50" s="10" t="inlineStr">
         <is>
           <t>ปกติ: 08:00 – 16:00 (8 ชม.)
 พีค: 07:30 – 17:00 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
+      <c r="F50" s="8" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="G46" s="8" t="inlineStr">
+      <c r="G50" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H46" s="8" t="inlineStr">
+      <c r="H50" s="8" t="inlineStr">
         <is>
           <t>42 – 48 ชม./wk</t>
         </is>
       </c>
-      <c r="I46" s="8" t="inlineStr">
+      <c r="I50" s="8" t="inlineStr">
         <is>
           <t>$100</t>
         </is>
       </c>
-      <c r="J46" s="10" t="inlineStr">
+      <c r="J50" s="10" t="inlineStr">
         <is>
           <t>อาณาจักรโรงแรมและรีสอร์ต Ruby’s Inn หน้าปากทาง Bryce Canyon NP, หอพักพนักงานใกล้ที่ทำงาน</t>
         </is>
       </c>
-      <c r="K46" s="10" t="inlineStr">
+      <c r="K50" s="10" t="inlineStr">
         <is>
           <t>🥩 Cowboy’s Buffet &amp; Steak Room (ในเครือ): Busser/Steward 17:00-22:30 น. (ขอ OT ในเครือ $22.50/ชม.)</t>
         </is>
       </c>
-      <c r="L46" s="10" t="inlineStr">
+      <c r="L50" s="10" t="inlineStr">
         <is>
           <t>🤠 Ebenezer’s Barn &amp; Grill: Food Runner งานดินเนอร์โชว์คาวบอย 18:00-22:00 น. (ได้ส่วนแบ่งทิป)</t>
         </is>
       </c>
-      <c r="M46" s="10" t="inlineStr">
+      <c r="M50" s="10" t="inlineStr">
         <is>
           <t>🛒 Ruby’s General Store &amp; Diner: แคชเชียร์/ผู้ช่วยครัว 17:00-21:30 น. ($15/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>Tier A - Utah (UT)</t>
         </is>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>Park City Mountain Resort (Vail Resorts - Park City)</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>OEG, Acadex</t>
-        </is>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>OEG, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Mountain Host / Housekeeping / F&amp;B</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E51" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 08:30 – 16:30 (8 ชม.)
 พีค: 08:00 – 17:30 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>ฐาน $17.50 / OT $26.25</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H47" s="5" t="inlineStr">
+      <c r="H51" s="5" t="inlineStr">
         <is>
           <t>42 – 48 ชม./wk</t>
         </is>
       </c>
-      <c r="I47" s="5" t="inlineStr">
+      <c r="I51" s="5" t="inlineStr">
         <is>
           <t>$150</t>
         </is>
       </c>
-      <c r="J47" s="7" t="inlineStr">
+      <c r="J51" s="7" t="inlineStr">
         <is>
           <t>สกีรีสอร์ตและเมืองภูเขาที่ใหญ่ที่สุดในสหรัฐฯ, ระบบรถเมล์ฟรีทั้งเมือง Park City Transit</t>
         </is>
       </c>
-      <c r="K47" s="7" t="inlineStr">
+      <c r="K51" s="7" t="inlineStr">
         <is>
           <t>🥩 High West Distillery &amp; Saloon (Main Street): Barback/Busser โรงกลั่นวิสกี้ดัง 17:30-23:30 น. (ทิปสด $80-$140/คืน)</t>
         </is>
       </c>
-      <c r="L47" s="7" t="inlineStr">
+      <c r="L51" s="7" t="inlineStr">
         <is>
           <t>🍕 Red Banjo Pizza (Historic Main St): ล้างจาน/ผู้ช่วยครัว 18:00-23:00 น. ($16/ชม. + ทิป)</t>
         </is>
       </c>
-      <c r="M47" s="7" t="inlineStr">
+      <c r="M51" s="7" t="inlineStr">
         <is>
           <t>🛒 Freshies Lobster Co. / Local Cafes: Food Runner 17:00-21:30 น. ($15/ชม. + ทิป)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Tier A - Maine (ME)</t>
         </is>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>Bar Harbor Grand Hotel / Harborside Hotel</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>Acadex, OEG, Higher</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>Acadex, OEG, Higher, IEO</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
         <is>
           <t>Housekeeping / Laundry</t>
         </is>
       </c>
-      <c r="E48" s="10" t="inlineStr">
+      <c r="E52" s="10" t="inlineStr">
         <is>
           <t>ปกติ: 08:00 – 16:00 (8 ชม.)
 พีค: 07:30 – 17:00 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr">
+      <c r="F52" s="8" t="inlineStr">
         <is>
           <t>ฐาน $16.50 / OT $24.75</t>
         </is>
       </c>
-      <c r="G48" s="8" t="inlineStr">
+      <c r="G52" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H48" s="8" t="inlineStr">
+      <c r="H52" s="8" t="inlineStr">
         <is>
           <t>44 – 50 ชม./wk</t>
         </is>
       </c>
-      <c r="I48" s="8" t="inlineStr">
+      <c r="I52" s="8" t="inlineStr">
         <is>
           <t>$130</t>
         </is>
       </c>
-      <c r="J48" s="10" t="inlineStr">
+      <c r="J52" s="10" t="inlineStr">
         <is>
           <t>เมืองตากอากาศชายทะเล Bar Harbor &amp; อุทยาน Acadia NP, รถบัส Island Explorer ฟรี</t>
         </is>
       </c>
-      <c r="K48" s="10" t="inlineStr">
+      <c r="K52" s="10" t="inlineStr">
         <is>
           <t>🦞 Stewman’s Lobster Pound (ริมทะเล): Busser/Barback ร้านกุ้งล็อบสเตอร์ 17:30-23:00 น. ($13/ชม. + ทิปสด $60-$120/คืน)</t>
         </is>
       </c>
-      <c r="L48" s="10" t="inlineStr">
+      <c r="L52" s="10" t="inlineStr">
         <is>
           <t>🍺 Geddy’s Down Under / The Chart Room: Busser/Runner 18:00-23:30 น. (ทิปสดแน่นมาก)</t>
         </is>
       </c>
-      <c r="M48" s="10" t="inlineStr">
+      <c r="M52" s="10" t="inlineStr">
         <is>
           <t>🍦 Ben &amp; Bill’s Chocolate Emporium: พนักงานตักไอศกรีม/แคชเชียร์ 17:00-22:00 น. ($15.50/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Tier A - Maine (ME)</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>Cliff House Maine (Cape Neddick / Ogunquit)</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>Higher, Acadex</t>
-        </is>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Higher, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>Housekeeping / Culinary / Stewarding</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="E53" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 08:00 – 16:30 (8 ชม.)
 พีค: 07:30 – 17:30 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F53" s="5" t="inlineStr">
         <is>
           <t>ฐาน $17.00 / OT $25.50</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H49" s="5" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
         <is>
           <t>42 – 48 ชม./wk</t>
         </is>
       </c>
-      <c r="I49" s="5" t="inlineStr">
+      <c r="I53" s="5" t="inlineStr">
         <is>
           <t>$135</t>
         </is>
       </c>
-      <c r="J49" s="7" t="inlineStr">
+      <c r="J53" s="7" t="inlineStr">
         <is>
           <t>รีสอร์ตหรูบนหน้าผาริมมหาสมุทรแอตแลนติก แขกไฮเอนด์ระดับมหาเศรษฐีบอสตันและนิวยอร์ก</t>
         </is>
       </c>
-      <c r="K49" s="7" t="inlineStr">
+      <c r="K53" s="7" t="inlineStr">
         <is>
           <t>🦞 The Tiller Restaurant (ในรีสอร์ต): Busser ร้าน Fine Dining วิวมหาสมุทร 17:30-23:00 น. (ทิปสด $70-$130/คืน)</t>
         </is>
       </c>
-      <c r="L49" s="7" t="inlineStr">
+      <c r="L53" s="7" t="inlineStr">
         <is>
           <t>🍺 Nubb’s Lobster Shack (ในรีสอร์ต): Food Runner/Barback 17:00-22:30 น. (ขอ OT ในรีสอร์ต $25.50)</t>
         </is>
       </c>
-      <c r="M49" s="7" t="inlineStr">
+      <c r="M53" s="7" t="inlineStr">
         <is>
           <t>🍦 Ogunquit Beach Cafes: ผู้ช่วยครัว/บริการรอบเย็น</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Tier A - Maine (ME)</t>
         </is>
       </c>
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B54" s="9" t="inlineStr">
         <is>
           <t>The Nonantum Resort (Kennebunkport, ME)</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>Higher, Acadex</t>
-        </is>
-      </c>
-      <c r="D50" s="9" t="inlineStr">
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Higher, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
         <is>
           <t>Housekeeping / Banquet / F&amp;B</t>
         </is>
       </c>
-      <c r="E50" s="10" t="inlineStr">
+      <c r="E54" s="10" t="inlineStr">
         <is>
           <t>ปกติ: 08:00 – 16:00 (8 ชม.)
 พีค: 07:30 – 17:00 (9.5 ชม.)</t>
         </is>
       </c>
-      <c r="F50" s="8" t="inlineStr">
+      <c r="F54" s="8" t="inlineStr">
         <is>
           <t>ฐาน $16.50 / OT $24.75</t>
         </is>
       </c>
-      <c r="G50" s="8" t="inlineStr">
+      <c r="G54" s="8" t="inlineStr">
         <is>
           <t>$20 - $50</t>
         </is>
       </c>
-      <c r="H50" s="8" t="inlineStr">
+      <c r="H54" s="8" t="inlineStr">
         <is>
           <t>42 – 48 ชม./wk</t>
         </is>
       </c>
-      <c r="I50" s="8" t="inlineStr">
+      <c r="I54" s="8" t="inlineStr">
         <is>
           <t>$125</t>
         </is>
       </c>
-      <c r="J50" s="10" t="inlineStr">
+      <c r="J54" s="10" t="inlineStr">
         <is>
           <t>รีสอร์ตตากอากาศริมน้ำประวัติศาสตร์ เมืองของประธานาธิบดีบุช, หอพักพนักงาน Kennebunkport</t>
         </is>
       </c>
-      <c r="K50" s="10" t="inlineStr">
+      <c r="K54" s="10" t="inlineStr">
         <is>
           <t>🦞 The Clam Shack (สะพาน Kennebunkport): ล้างจาน/ทอดซีฟู้ดร้านดัง 17:30-22:30 น. ($16/ชม. + ทิป)</t>
         </is>
       </c>
-      <c r="L50" s="10" t="inlineStr">
+      <c r="L54" s="10" t="inlineStr">
         <is>
           <t>🥩 Ocean Restaurant: Busser ร้านอาหารหรูริมน้ำ 18:00-23:00 น. (ทิปสด $60-$100/คืน)</t>
         </is>
       </c>
-      <c r="M50" s="10" t="inlineStr">
+      <c r="M54" s="10" t="inlineStr">
         <is>
           <t>🍦 Rococo Artisan Ice Cream: ตักไอศกรีม 17:00-22:00 น. ($15/ชม.)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>Tier A - Ohio (OH)</t>
         </is>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>Cedar Point Amusement Park &amp; Resorts (Sandusky)</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>OEG, IEE Thailand</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>OEG, IEE Thailand, IEO</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Ride Operator / Food Service</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 10:00 – 18:30 (8 ชม.)
 พีค: 09:30 – 22:30 (12 ชม. สวนสนุกปิดดึก)</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t>ฐาน $14.50 / OT $21.75</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H51" s="5" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>46 – 52 ชม./wk</t>
         </is>
       </c>
-      <c r="I51" s="5" t="inlineStr">
+      <c r="I55" s="5" t="inlineStr">
         <is>
           <t>$80 (ถูกสุด)</t>
         </is>
       </c>
-      <c r="J51" s="7" t="inlineStr">
+      <c r="J55" s="7" t="inlineStr">
         <is>
           <t>สวนสนุกเครื่องเล่นระดับโลก, หอพักราคาถูกที่สุดในอเมริกา ($80/wk), รถบัสรับส่งฟรี, เล่นสวนสนุกฟรี</t>
         </is>
       </c>
-      <c r="K51" s="7" t="inlineStr">
+      <c r="K55" s="7" t="inlineStr">
         <is>
           <t>🏨 Hotel Breakers / Castaway Bay (ในสวนสนุก): ล้างจาน/แม่บ้านกะค่ำ 19:00-00:00 น. (ขอ OT ในสวนสนุก $21.75/ชม.)</t>
         </is>
       </c>
-      <c r="L51" s="7" t="inlineStr">
+      <c r="L55" s="7" t="inlineStr">
         <is>
           <t>🍖 Famous Dave’s BBQ (Cedar Point Marina): Busser/Dishwasher 18:30-23:30 น. ($13/ชม. + ทิปสด)</t>
         </is>
       </c>
-      <c r="M51" s="7" t="inlineStr">
+      <c r="M55" s="7" t="inlineStr">
         <is>
           <t>🐴 Thirsty Pony / Kalahari Sandusky: Barback/Busser ร้านอาหารใกล้เคียง 19:00-00:30 น.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>Tier A - Ohio (OH)</t>
         </is>
       </c>
-      <c r="B52" s="9" t="inlineStr">
+      <c r="B56" s="9" t="inlineStr">
         <is>
           <t>Kings Island Amusement Park (Mason / Cincinnati)</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>OEG, IEE Thailand</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>OEG, IEE Thailand, IEO</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
         <is>
           <t>Ride Operator / Park Services / Culinary</t>
         </is>
       </c>
-      <c r="E52" s="10" t="inlineStr">
+      <c r="E56" s="10" t="inlineStr">
         <is>
           <t>ปกติ: 10:00 – 18:30 (8 ชม.)
 พีค: 09:30 – 22:30 (12 ชม.)</t>
         </is>
       </c>
-      <c r="F52" s="8" t="inlineStr">
+      <c r="F56" s="8" t="inlineStr">
         <is>
           <t>ฐาน $14.50 / OT $21.75</t>
         </is>
       </c>
-      <c r="G52" s="8" t="inlineStr">
+      <c r="G56" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H52" s="8" t="inlineStr">
+      <c r="H56" s="8" t="inlineStr">
         <is>
           <t>44 – 50 ชม./wk</t>
         </is>
       </c>
-      <c r="I52" s="8" t="inlineStr">
+      <c r="I56" s="8" t="inlineStr">
         <is>
           <t>$90</t>
         </is>
       </c>
-      <c r="J52" s="10" t="inlineStr">
+      <c r="J56" s="10" t="inlineStr">
         <is>
           <t>สวนสนุกชั้นนำเครือ Cedar Fair ใกล้เมือง Cincinnati, หอพักพนักงาน + รถรับส่งฟรี</t>
         </is>
       </c>
-      <c r="K52" s="10" t="inlineStr">
+      <c r="K56" s="10" t="inlineStr">
         <is>
           <t>🍕 Mason Local Pizzerias &amp; Diners: ล้างจาน/ผู้ช่วยครัวรอบดึก 19:00-00:00 น. ($14.50/ชม.)</t>
         </is>
       </c>
-      <c r="L52" s="10" t="inlineStr">
+      <c r="L56" s="10" t="inlineStr">
         <is>
           <t>🍦 Greaters Ice Cream: พนักงานตักไอศกรีมชื่อดัง 19:00-23:00 น. ($14.50/ชม.)</t>
         </is>
       </c>
-      <c r="M52" s="10" t="inlineStr">
+      <c r="M56" s="10" t="inlineStr">
         <is>
           <t>🏨 Great Wolf Lodge Mason (ข้างๆ สวนสนุก): แม่บ้าน/ผู้ช่วยครัวกะค่ำ (ขอทำเพิ่มได้)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Tier A - Colorado (CO)</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>YMCA of the Rockies (Estes Park Center)</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>Higher, IEE, Acadex</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Higher, IEE, Acadex, IEO</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Housekeeping / Food Service</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr">
+      <c r="E57" s="7" t="inlineStr">
         <is>
           <t>ปกติ: 07:30 – 15:30 (8 ชม.)
 พีค: 07:00 – 16:30 (9 ชม.)</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr">
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H53" s="5" t="inlineStr">
+      <c r="H57" s="5" t="inlineStr">
         <is>
           <t>42 – 48 ชม./wk</t>
         </is>
       </c>
-      <c r="I53" s="5" t="inlineStr">
+      <c r="I57" s="5" t="inlineStr">
         <is>
           <t>$110 (รวมกิน)</t>
         </is>
       </c>
-      <c r="J53" s="7" t="inlineStr">
+      <c r="J57" s="7" t="inlineStr">
         <is>
           <t>แคมป์รีสอร์ตกลางเทือกเขา Rocky Mountain NP, หอพัก+อาหารบุฟเฟต์ 3 มื้อ, รถชัตเติลบัสเข้าเมืองฟรี</t>
         </is>
       </c>
-      <c r="K53" s="7" t="inlineStr">
+      <c r="K57" s="7" t="inlineStr">
         <is>
           <t>🏨 The Stanley Hotel (โรงแรมประวัติศาสตร์ The Shining): Busser/Steward ร้านอาหารหรู 17:30-23:00 น. (ทิปสด $50-$90)</t>
         </is>
       </c>
-      <c r="L53" s="7" t="inlineStr">
+      <c r="L57" s="7" t="inlineStr">
         <is>
           <t>🍔 Penelope’s Old Time Burgers: ผู้ช่วยครัว/ทอดเบอร์เกอร์ 17:00-21:30 น. ($15/ชม. + กินฟรี)</t>
         </is>
       </c>
-      <c r="M53" s="7" t="inlineStr">
+      <c r="M57" s="7" t="inlineStr">
         <is>
           <t>🍺 Estes Park Brewery / Rock Cut Brewing: ล้างแก้ว/ผู้ช่วยบาร์ 18:00-22:30 น. ($15/ชม.)</t>
         </is>

</xml_diff>

<commit_message>
Removed 12-week simulator sheet as requested
</commit_message>
<xml_diff>
--- a/Work_and_Travel_Master_Job_Database_2027.xlsx
+++ b/Work_and_Travel_Master_Job_Database_2027.xlsx
@@ -9,8 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top Employers (Summer Only)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier S-A Summer Jobs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summer 12-Week Simulator" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summer Agency Directory" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summer Agency Directory" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="#,##0฿"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -94,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -125,12 +121,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8543,834 +8533,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="79" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="39" customWidth="1" min="15" max="15"/>
-    <col width="31" customWidth="1" min="16" max="16"/>
-    <col width="35" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>สัปดาห์ (Summer Week)</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>ช่วงวันที่ (Summer Timeline)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>สถานการณ์ &amp; รายละเอียดกะงานซัมเมอร์</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ชม. งานหลัก (ชม.)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ชม. งานสอง (ชม.)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>รวม ชม./สัปดาห์</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>รายรับงานหลัก ($)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>รายรับงานสอง ($)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>เงินทิปสด ($)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>รายรับรวมรายสัปดาห์ ($)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>รายรับรวม (บาท)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>หักภาษี Fed 10% ($)</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>หักหอพัก/EDR ($)</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>หักของใช้ส่วนตัว ($)</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>เงินสดสุทธิสัปดาห์นั้น ($)</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>เงินสดสะสมคงเหลือ ($)</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>เงินสดสะสมคงเหลือ (บาท)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Week 1</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>7 พ.ค. - 14 พ.ค.</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>เดินทางถึง, ปฐมนิเทศ, อบรม, ทำ SSN ที่แฟร์แบงก์ส</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>32</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>32</v>
-      </c>
-      <c r="G2" s="11" t="n">
-        <v>512</v>
-      </c>
-      <c r="H2" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" s="11" t="n">
-        <v>512</v>
-      </c>
-      <c r="K2" s="12" t="n">
-        <v>16819</v>
-      </c>
-      <c r="L2" s="11" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="M2" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N2" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O2" s="11" t="n">
-        <v>330.8</v>
-      </c>
-      <c r="P2" s="11" t="n">
-        <v>330.8</v>
-      </c>
-      <c r="Q2" s="12" t="n">
-        <v>10867</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Week 2</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>15 พ.ค. - 21 พ.ค.</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>เปิดซีซันซัมเมอร์, เรือสำราญรอบแรกเข้า, สมัครงาน 2</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="G3" s="11" t="n">
-        <v>608</v>
-      </c>
-      <c r="H3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="11" t="n">
-        <v>608</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>19973</v>
-      </c>
-      <c r="L3" s="11" t="n">
-        <v>60.8</v>
-      </c>
-      <c r="M3" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N3" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O3" s="11" t="n">
-        <v>417.2</v>
-      </c>
-      <c r="P3" s="11" t="n">
-        <v>748</v>
-      </c>
-      <c r="Q3" s="12" t="n">
-        <v>24572</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Week 3</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>22 พ.ค. - 28 พ.ค. (Memorial Day)</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>วันหยุด Memorial Day เปิดซัมเมอร์เต็มรูปแบบ งานสองเริ่มทำ</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>48</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>832</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>150</v>
-      </c>
-      <c r="I4" s="11" t="n">
-        <v>60</v>
-      </c>
-      <c r="J4" s="11" t="n">
-        <v>1042</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>34230</v>
-      </c>
-      <c r="L4" s="11" t="n">
-        <v>104.2</v>
-      </c>
-      <c r="M4" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N4" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O4" s="11" t="n">
-        <v>807.8</v>
-      </c>
-      <c r="P4" s="11" t="n">
-        <v>1555.8</v>
-      </c>
-      <c r="Q4" s="12" t="n">
-        <v>51108</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Week 4</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>29 พ.ค. - 4 มิ.ย.</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>รถไฟทัวร์แน่น, เข้าที่เต็มตัว, งานสอง Barback 4 วัน</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>54</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>68</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>976</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>120</v>
-      </c>
-      <c r="J5" s="11" t="n">
-        <v>1306</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>42902</v>
-      </c>
-      <c r="L5" s="11" t="n">
-        <v>130.6</v>
-      </c>
-      <c r="M5" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N5" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O5" s="11" t="n">
-        <v>1045.4</v>
-      </c>
-      <c r="P5" s="11" t="n">
-        <v>2601.2</v>
-      </c>
-      <c r="Q5" s="12" t="n">
-        <v>85449</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Week 5</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>5 มิ.ย. - 11 มิ.ย.</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>ช่วง Midnight Sun สว่าง 24 ชม. แขกแน่นตลอดคืน</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>56</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>70</v>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>1024</v>
-      </c>
-      <c r="H6" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="I6" s="11" t="n">
-        <v>140</v>
-      </c>
-      <c r="J6" s="11" t="n">
-        <v>1374</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>45136</v>
-      </c>
-      <c r="L6" s="11" t="n">
-        <v>137.4</v>
-      </c>
-      <c r="M6" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N6" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O6" s="11" t="n">
-        <v>1106.6</v>
-      </c>
-      <c r="P6" s="11" t="n">
-        <v>3707.8</v>
-      </c>
-      <c r="Q6" s="12" t="n">
-        <v>121801</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Week 6</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>12 มิ.ย. - 18 มิ.ย.</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>PEAK ซัมเมอร์ เรือสำราญและรถไฟเข้าเต็มพิกัด</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>56</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>70</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>1024</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="I7" s="11" t="n">
-        <v>140</v>
-      </c>
-      <c r="J7" s="11" t="n">
-        <v>1374</v>
-      </c>
-      <c r="K7" s="12" t="n">
-        <v>45136</v>
-      </c>
-      <c r="L7" s="11" t="n">
-        <v>137.4</v>
-      </c>
-      <c r="M7" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N7" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O7" s="11" t="n">
-        <v>1106.6</v>
-      </c>
-      <c r="P7" s="11" t="n">
-        <v>4814.4</v>
-      </c>
-      <c r="Q7" s="12" t="n">
-        <v>158153</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Week 7</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>19 มิ.ย. - 25 มิ.ย.</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>ฝนตกในหุบเขา/รถไฟดีเลย์ ร่างกายเริ่มล้า พักผ่อน</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>44</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>56</v>
-      </c>
-      <c r="G8" s="11" t="n">
-        <v>736</v>
-      </c>
-      <c r="H8" s="11" t="n">
-        <v>180</v>
-      </c>
-      <c r="I8" s="11" t="n">
-        <v>80</v>
-      </c>
-      <c r="J8" s="11" t="n">
-        <v>996</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>32719</v>
-      </c>
-      <c r="L8" s="11" t="n">
-        <v>99.59999999999999</v>
-      </c>
-      <c r="M8" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N8" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O8" s="11" t="n">
-        <v>766.4</v>
-      </c>
-      <c r="P8" s="11" t="n">
-        <v>5580.8</v>
-      </c>
-      <c r="Q8" s="12" t="n">
-        <v>183330</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Week 8</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>26 มิ.ย. - 4 ก.ค. (4th of July PEAK)</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>วันชาติอเมริกา PEAK ที่สุดในรอบปี แขกล้น ทิปมหาศาล</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>73</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1072</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>225</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>160</v>
-      </c>
-      <c r="J9" s="11" t="n">
-        <v>1457</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>47862</v>
-      </c>
-      <c r="L9" s="11" t="n">
-        <v>145.7</v>
-      </c>
-      <c r="M9" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N9" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O9" s="11" t="n">
-        <v>1181.3</v>
-      </c>
-      <c r="P9" s="11" t="n">
-        <v>6762.1</v>
-      </c>
-      <c r="Q9" s="12" t="n">
-        <v>222135</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Week 9</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>5 ก.ค. - 15 ก.ค.</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>ช่วงพีคต่อเนื่อง นักท่องเที่ยวครอบครัวสหรัฐฯ แน่น</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>52</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>64</v>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>928</v>
-      </c>
-      <c r="H10" s="11" t="n">
-        <v>180</v>
-      </c>
-      <c r="I10" s="11" t="n">
-        <v>120</v>
-      </c>
-      <c r="J10" s="11" t="n">
-        <v>1228</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>40340</v>
-      </c>
-      <c r="L10" s="11" t="n">
-        <v>122.8</v>
-      </c>
-      <c r="M10" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N10" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O10" s="11" t="n">
-        <v>975.2</v>
-      </c>
-      <c r="P10" s="11" t="n">
-        <v>7737.3</v>
-      </c>
-      <c r="Q10" s="12" t="n">
-        <v>254171</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Week 10</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>16 ก.ค. - 31 ก.ค.</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>เข้าสู่ปลายซัมเมอร์ นักศึกษาฝรั่งเริ่มทยอยกลับ</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>48</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>832</v>
-      </c>
-      <c r="H11" s="11" t="n">
-        <v>150</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="J11" s="11" t="n">
-        <v>1082</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>35544</v>
-      </c>
-      <c r="L11" s="11" t="n">
-        <v>108.2</v>
-      </c>
-      <c r="M11" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N11" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O11" s="11" t="n">
-        <v>843.8</v>
-      </c>
-      <c r="P11" s="11" t="n">
-        <v>8581.1</v>
-      </c>
-      <c r="Q11" s="12" t="n">
-        <v>281890</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Week 11</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>1 ส.ค. - 15 ส.ค.</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>ใบไม้เริ่มเปลี่ยนสี ทัวร์ซา ปิดห้องพักบางโซน</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>44</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>52</v>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>736</v>
-      </c>
-      <c r="H12" s="11" t="n">
-        <v>120</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>60</v>
-      </c>
-      <c r="J12" s="11" t="n">
-        <v>916</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>30091</v>
-      </c>
-      <c r="L12" s="11" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="M12" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N12" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O12" s="11" t="n">
-        <v>694.4</v>
-      </c>
-      <c r="P12" s="11" t="n">
-        <v>9275.5</v>
-      </c>
-      <c r="Q12" s="12" t="n">
-        <v>304701</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Week 12</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>16 ส.ค. - 7 ก.ย. (Wrap Up)</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>สัปดาห์สุดท้าย เคลียร์ห้อง ปิดซีซันซัมเมอร์ คืนมัดจำ</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="G13" s="11" t="n">
-        <v>576</v>
-      </c>
-      <c r="H13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="11" t="n">
-        <v>576</v>
-      </c>
-      <c r="K13" s="12" t="n">
-        <v>18922</v>
-      </c>
-      <c r="L13" s="11" t="n">
-        <v>57.6</v>
-      </c>
-      <c r="M13" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="N13" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="O13" s="11" t="n">
-        <v>388.4</v>
-      </c>
-      <c r="P13" s="11" t="n">
-        <v>9663.9</v>
-      </c>
-      <c r="Q13" s="12" t="n">
-        <v>317459</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Update GTLC housing to  (Room and Board bundle)
</commit_message>
<xml_diff>
--- a/Work_and_Travel_Master_Job_Database_2027.xlsx
+++ b/Work_and_Travel_Master_Job_Database_2027.xlsx
@@ -1073,12 +1073,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>$0 (ฟรี!)</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>หอพักฟรี 100%! + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), ส่วนลด 40%, บัตรผ่าน 2 อุทยานฟรี</t>
+          <t>หอพัก + อาหารบุฟเฟต์ 3 มื้อ EDR ตักไม่อั้น 7 วัน ($105/wk), ส่วนลดซื้อของ 40%, เข้าอุทยาน Grand Teton &amp; Yellowstone ฟรี</t>
         </is>
       </c>
     </row>
@@ -1131,12 +1131,12 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>$0 (ฟรี!)</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>หอพักฟรี 100%! + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), หมู่บ้านริมทะเลสาบ Jackson Lake</t>
+          <t>หอพัก + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), หมู่บ้านริมทะเลสาบ Jackson Lake สวยที่สุดในซัมเมอร์</t>
         </is>
       </c>
     </row>
@@ -4775,12 +4775,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>$0 (ฟรี!)</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>หอพักฟรี 100%! + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), ส่วนลด 40%, บัตรผ่าน 2 อุทยานฟรี</t>
+          <t>หอพัก + อาหารบุฟเฟต์ 3 มื้อ EDR ตักไม่อั้น 7 วัน ($105/wk), ส่วนลดซื้อของ 40%, เข้าอุทยาน Grand Teton &amp; Yellowstone ฟรี</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -4848,12 +4848,12 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>$0 (ฟรี!)</t>
+          <t>$105</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>หอพักฟรี 100%! + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), หมู่บ้านริมทะเลสาบ Jackson Lake</t>
+          <t>หอพัก + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), หมู่บ้านริมทะเลสาบ Jackson Lake สวยที่สุดในซัมเมอร์</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Annotate all jobs offering included/free meals with (รวมกิน) in housing column
</commit_message>
<xml_diff>
--- a/Work_and_Travel_Master_Job_Database_2027.xlsx
+++ b/Work_and_Travel_Master_Job_Database_2027.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K52" s="10" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -7841,7 +7841,7 @@
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>$105</t>
+          <t>$105 (รวมกิน)</t>
         </is>
       </c>
       <c r="K52" s="10" t="inlineStr">

</xml_diff>